<commit_message>
chore(data-release): publish site data 2026-10-25 02:00:39 UTC
</commit_message>
<xml_diff>
--- a/countries/kr/2026-2029.xlsx
+++ b/countries/kr/2026-2029.xlsx
@@ -82408,13 +82408,13 @@
         </is>
       </c>
       <c r="N604" t="n">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="O604" t="n">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="R604" t="n">
-        <v>0.8372030070781639</v>
+        <v>0.8430169168495401</v>
       </c>
       <c r="AA604" t="inlineStr">
         <is>
@@ -85518,13 +85518,13 @@
         </is>
       </c>
       <c r="N627" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O627" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R627" t="n">
-        <v>0.06007706763755342</v>
+        <v>0.05813909771376138</v>
       </c>
       <c r="AA627" t="inlineStr">
         <is>
@@ -89031,7 +89031,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>96107</v>
+        <v>96109</v>
       </c>
     </row>
     <row r="16">

</xml_diff>